<commit_message>
Rename 광접속함체→광기구, update part format SP-→GK-, SPFC→GKFC
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM 자료/A11-D1-0000/A11-D1-0000_27형_기본.xlsx
+++ b/BOM 자료/A11-D1-0000/A11-D1-0000_27형_기본.xlsx
@@ -403,7 +403,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>회사명 : (주)샘플전자 / A11-D1-0000 / 27형 함체 (SPFC-D1) [기본]</v>
+        <v>회사명 : (주)샘플전자 / A11-D1-0000 / 27형 함체 (GKFC-D1) [기본]</v>
       </c>
       <c r="B1" t="str">
         <v/>
@@ -432,7 +432,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SP-00001</v>
+        <v>GK-00001</v>
       </c>
       <c r="B2" t="str">
         <v>품목명</v>
@@ -461,10 +461,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>SP-00105</v>
+        <v>GK-00105</v>
       </c>
       <c r="B3" t="str">
-        <v>SPFC-D1 상판 (SPFC-D1 TOP)</v>
+        <v>GKFC-D1 상판 (GKFC-D1 TOP)</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -490,10 +490,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>SP-00106</v>
+        <v>GK-00106</v>
       </c>
       <c r="B4" t="str">
-        <v>SPFC-D1 하판 (SPFC-D1 BOTTOM)</v>
+        <v>GKFC-D1 하판 (GKFC-D1 BOTTOM)</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -519,7 +519,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>SP-00068</v>
+        <v>GK-00068</v>
       </c>
       <c r="B5" t="str">
         <v>OFC 광케이블 고정대 B형 (OFC OPTICAL CABLE FIXTURE B TYPE)</v>
@@ -548,7 +548,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SP-00107</v>
+        <v>GK-00107</v>
       </c>
       <c r="B6" t="str">
         <v>OFC 광케이블 고정대 C형 (OFC OPTICAL CABLE FIXTURE C TYPE)</v>
@@ -577,10 +577,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>SP-00108</v>
+        <v>GK-00108</v>
       </c>
       <c r="B7" t="str">
-        <v>SPFC-D1 트레이 (SPFC-D1 TRAY)</v>
+        <v>GKFC-D1 트레이 (GKFC-D1 TRAY)</v>
       </c>
       <c r="C7" t="str">
         <v/>
@@ -606,7 +606,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>SP-00109</v>
+        <v>GK-00109</v>
       </c>
       <c r="B8" t="str">
         <v>트레이 OZ_리본용 12슬롯 (SPLICE HOLDER_RIBBON TYPE 12 SLOT)</v>
@@ -635,10 +635,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SP-00110</v>
+        <v>GK-00110</v>
       </c>
       <c r="B9" t="str">
-        <v>SPFC 인입구 마개 OD8 (SPFC LEADING IN ROD OD8)</v>
+        <v>GKFC 인입구 마개 OD8 (GKFC LEADING IN ROD OD8)</v>
       </c>
       <c r="C9" t="str">
         <v>∅8mm*L40mm</v>
@@ -664,10 +664,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>SP-00111</v>
+        <v>GK-00111</v>
       </c>
       <c r="B10" t="str">
-        <v>SPFC 인입구 마개 OD15 (SPFC LEADING IN ROD OD15)</v>
+        <v>GKFC 인입구 마개 OD15 (GKFC LEADING IN ROD OD15)</v>
       </c>
       <c r="C10" t="str">
         <v>15mm</v>
@@ -693,10 +693,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>SP-00112</v>
+        <v>GK-00112</v>
       </c>
       <c r="B11" t="str">
-        <v>SPFC 인입구 마개 OD23 (SPFC LEADING IN ROD OD23)</v>
+        <v>GKFC 인입구 마개 OD23 (GKFC LEADING IN ROD OD23)</v>
       </c>
       <c r="C11" t="str">
         <v>23mm</v>
@@ -722,7 +722,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>SP-00069</v>
+        <v>GK-00069</v>
       </c>
       <c r="B12" t="str">
         <v>OFC 스패츌라 (OFC SPATULAR)</v>
@@ -751,7 +751,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>SP-00050</v>
+        <v>GK-00050</v>
       </c>
       <c r="B13" t="str">
         <v>압축 스프링 ID6.5*WD0.5*CL5*L35 (COMPRESSION SPRING ID6.5*WD0.5*CL5*L35)</v>
@@ -780,10 +780,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SP-00113</v>
+        <v>GK-00113</v>
       </c>
       <c r="B14" t="str">
-        <v>SPFC-D1 접지바 (SPFC-D1 GROUND BAR)</v>
+        <v>GKFC-D1 접지바 (GKFC-D1 GROUND BAR)</v>
       </c>
       <c r="C14" t="str">
         <v/>
@@ -809,10 +809,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SP-00114</v>
+        <v>GK-00114</v>
       </c>
       <c r="B15" t="str">
-        <v>SPFC-C1 인장선 고정철판 (SPFC-C1 TENSION LINE FIXTURE)</v>
+        <v>GKFC-C1 인장선 고정철판 (GKFC-C1 TENSION LINE FIXTURE)</v>
       </c>
       <c r="C15" t="str">
         <v>ㄷ자</v>
@@ -838,10 +838,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SP-00115</v>
+        <v>GK-00115</v>
       </c>
       <c r="B16" t="str">
-        <v>SPFC-D1 트레이 스토퍼 (SPFC-D1 TRAY STOPPER)</v>
+        <v>GKFC-D1 트레이 스토퍼 (GKFC-D1 TRAY STOPPER)</v>
       </c>
       <c r="C16" t="str">
         <v/>
@@ -867,10 +867,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SP-00064</v>
+        <v>GK-00064</v>
       </c>
       <c r="B17" t="str">
-        <v>SPFC-B4 브라켓 (SPFC-B4 BRACKET)</v>
+        <v>GKFC-B4 브라켓 (GKFC-B4 BRACKET)</v>
       </c>
       <c r="C17" t="str">
         <v>가공형 브라켓</v>
@@ -896,7 +896,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SP-00055</v>
+        <v>GK-00055</v>
       </c>
       <c r="B18" t="str">
         <v>육각볼트 M6*L40_TAP10 (HEXAGON BOLT M6*L40_TAP10)</v>
@@ -925,7 +925,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SP-00116</v>
+        <v>GK-00116</v>
       </c>
       <c r="B19" t="str">
         <v>육각볼트 M6*L42_TAP10 (HEXAGON BOLT M6*L42_TAP10)</v>
@@ -954,7 +954,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SP-00051</v>
+        <v>GK-00051</v>
       </c>
       <c r="B20" t="str">
         <v>평와셔 M6*OD14*T1.5 (FLAT WASHER M6*OD14*T1.5)</v>
@@ -983,7 +983,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SP-00117</v>
+        <v>GK-00117</v>
       </c>
       <c r="B21" t="str">
         <v>접지볼트 M5*L16 (STUD BOLT M5*L16)</v>
@@ -1012,7 +1012,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SP-00118</v>
+        <v>GK-00118</v>
       </c>
       <c r="B22" t="str">
         <v>SUS 육각 너트 M5*OD8*L4 (SUS HEXAGON NUT M5*OD8*L4)</v>
@@ -1041,7 +1041,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SP-00081</v>
+        <v>GK-00081</v>
       </c>
       <c r="B23" t="str">
         <v>평와셔 M5*OD12*T0.5 (FLAT WASHER M5*OD12*T0.5)</v>
@@ -1070,7 +1070,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SP-00008</v>
+        <v>GK-00008</v>
       </c>
       <c r="B24" t="str">
         <v>오링 P-5 (O-RING P-5)</v>
@@ -1099,7 +1099,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SP-00119</v>
+        <v>GK-00119</v>
       </c>
       <c r="B25" t="str">
         <v>트러스 볼트 M5*L30 (TRUSS BOLT M5*L30)</v>
@@ -1128,7 +1128,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SP-00054</v>
+        <v>GK-00054</v>
       </c>
       <c r="B26" t="str">
         <v>트러스 볼트 M5*L35 (TRUSS BOLT M5*L35)</v>
@@ -1157,7 +1157,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SP-00120</v>
+        <v>GK-00120</v>
       </c>
       <c r="B27" t="str">
         <v>트러스 볼트 M5*L40 (TRUSS BOLT M5*L40)</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SP-00121</v>
+        <v>GK-00121</v>
       </c>
       <c r="B28" t="str">
         <v>2종 와셔붙이 볼트 M3*L10 (2 STAGE SEMS BOLT M3*L10)</v>
@@ -1215,7 +1215,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>SP-00122</v>
+        <v>GK-00122</v>
       </c>
       <c r="B29" t="str">
         <v>트러스 볼트 M5*L16 (TRUSS BOLT M5*L16)</v>
@@ -1244,7 +1244,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>SP-00011</v>
+        <v>GK-00011</v>
       </c>
       <c r="B30" t="str">
         <v>인서트 너트 M6*OD10*L10_Ni (INSERT NUT M6*OD10*L10_Ni)</v>
@@ -1273,7 +1273,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>SP-00123</v>
+        <v>GK-00123</v>
       </c>
       <c r="B31" t="str">
         <v>인서트 너트 M5*OD8*L10_Ni ( INSERT NUT M5*OD8*L10_Ni)</v>
@@ -1302,10 +1302,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>SP-00124</v>
+        <v>GK-00124</v>
       </c>
       <c r="B32" t="str">
-        <v>SPFC-D1 가스켓 (SPFC-D1 GASKET)</v>
+        <v>GKFC-D1 가스켓 (GKFC-D1 GASKET)</v>
       </c>
       <c r="C32" t="str">
         <v/>
@@ -1331,10 +1331,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>SP-00125</v>
+        <v>GK-00125</v>
       </c>
       <c r="B33" t="str">
-        <v>SPFC-C1 인입구 그로멧 ID8-12 (SPFC-C1 CABLE GROMMET ID8-12)</v>
+        <v>GKFC-C1 인입구 그로멧 ID8-12 (GKFC-C1 CABLE GROMMET ID8-12)</v>
       </c>
       <c r="C33" t="str">
         <v>B-C1,C2,D1 (19,24,27) / 8-12mm</v>
@@ -1360,10 +1360,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>SP-00126</v>
+        <v>GK-00126</v>
       </c>
       <c r="B34" t="str">
-        <v>SPFC-C1 인입구 그로멧 ID12-17 (SPFC-C1 CABLE GROMMET ID12-17)</v>
+        <v>GKFC-C1 인입구 그로멧 ID12-17 (GKFC-C1 CABLE GROMMET ID12-17)</v>
       </c>
       <c r="C34" t="str">
         <v>B-C1,C2,D1 (19,24,27) / 12-17mm</v>
@@ -1389,10 +1389,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>SP-00127</v>
+        <v>GK-00127</v>
       </c>
       <c r="B35" t="str">
-        <v>SPFC-D1 인입구 그로멧 ID23 (SPFC-D1 CABLE GROMMET ID23)</v>
+        <v>GKFC-D1 인입구 그로멧 ID23 (GKFC-D1 CABLE GROMMET ID23)</v>
       </c>
       <c r="C35" t="str">
         <v>B-D1 (27) / 23mm</v>
@@ -1418,13 +1418,13 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>SP-00128</v>
+        <v>GK-00128</v>
       </c>
       <c r="B36" t="str">
         <v>라벨 스티커 (별표, 트레이에 부착)</v>
       </c>
       <c r="C36" t="str">
-        <v>SPFC-D1 (NBG)</v>
+        <v>GKFC-D1 (NBG)</v>
       </c>
       <c r="D36" t="str">
         <v>-1</v>
@@ -1447,13 +1447,13 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>SP-00129</v>
+        <v>GK-00129</v>
       </c>
       <c r="B37" t="str">
         <v>라벨스티커 (고객A, 함체 상판 스티커)</v>
       </c>
       <c r="C37" t="str">
-        <v>SPFC-D1 (124*44)</v>
+        <v>GKFC-D1 (124*44)</v>
       </c>
       <c r="D37" t="str">
         <v>1</v>
@@ -1476,7 +1476,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>SP-00130</v>
+        <v>GK-00130</v>
       </c>
       <c r="B38" t="str">
         <v>사용설명서 (User manual)</v>
@@ -1505,10 +1505,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>SP-00131</v>
+        <v>GK-00131</v>
       </c>
       <c r="B39" t="str">
-        <v>SPFC-D1 트레이 커버 (SPFC-D1 TRAY COVER)</v>
+        <v>GKFC-D1 트레이 커버 (GKFC-D1 TRAY COVER)</v>
       </c>
       <c r="C39" t="str">
         <v/>
@@ -1534,7 +1534,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>SP-00132</v>
+        <v>GK-00132</v>
       </c>
       <c r="B40" t="str">
         <v>벨크로 L700 (Velcro Strap L700)</v>
@@ -1563,7 +1563,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>SP-00087</v>
+        <v>GK-00087</v>
       </c>
       <c r="B41" t="str">
         <v>지퍼백 W55*D80 (PLASTIC BAG W55*D80)</v>
@@ -1592,7 +1592,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>SP-00133</v>
+        <v>GK-00133</v>
       </c>
       <c r="B42" t="str">
         <v>지퍼백 W80*D100 (PLASTIC BAG W80*D100)</v>
@@ -1621,13 +1621,13 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>SP-00044</v>
+        <v>GK-00044</v>
       </c>
       <c r="B43" t="str">
         <v>진공 그리스(Grease)</v>
       </c>
       <c r="C43" t="str">
-        <v>5g, SPFC-B4, SPFC-B1, SPFC-B2</v>
+        <v>5g, GKFC-B4, GKFC-B1, GKFC-B2</v>
       </c>
       <c r="D43" t="str">
         <v>1</v>
@@ -1650,7 +1650,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>SP-00134</v>
+        <v>GK-00134</v>
       </c>
       <c r="B44" t="str">
         <v>보호튜브 ID8.5*OD9.5_6C_L600_청등녹적황자</v>
@@ -1679,7 +1679,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>SP-00042</v>
+        <v>GK-00042</v>
       </c>
       <c r="B45" t="str">
         <v>절연테이프 W19*L10000 (Insulation Tape W19*L10000)</v>
@@ -1708,7 +1708,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>SP-00004</v>
+        <v>GK-00004</v>
       </c>
       <c r="B46" t="str">
         <v>케이블 타이 L100 (CABLE TIE L100)</v>
@@ -1737,7 +1737,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>SP-00082</v>
+        <v>GK-00082</v>
       </c>
       <c r="B47" t="str">
         <v>케이블 타이 L200 (CABLE TIE L200)</v>
@@ -1766,7 +1766,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>SP-00047</v>
+        <v>GK-00047</v>
       </c>
       <c r="B48" t="str">
         <v>에어밸브 (AIR VALVE)</v>
@@ -1795,7 +1795,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>SP-00074</v>
+        <v>GK-00074</v>
       </c>
       <c r="B49" t="str">
         <v>지퍼백 W150*D200 (PLASTIC BAG W150*D200)</v>
@@ -1824,7 +1824,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>SP-00048</v>
+        <v>GK-00048</v>
       </c>
       <c r="B50" t="str">
         <v>SUS 지지봉 OD22.3*T0.9*L1000 (SUS Mounting Rod OD22.3*T0.9*L1000)</v>
@@ -1853,13 +1853,13 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>SP-00135</v>
+        <v>GK-00135</v>
       </c>
       <c r="B51" t="str">
         <v>트레이 선번 스티커 (Splice Tray KR L-24)</v>
       </c>
       <c r="C51" t="str">
-        <v>SPFC-C1/C2, ZOFC-D2</v>
+        <v>GKFC-C1/C2, ZOFC-D2</v>
       </c>
       <c r="D51" t="str">
         <v>4</v>
@@ -1882,10 +1882,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>SP-00136</v>
+        <v>GK-00136</v>
       </c>
       <c r="B52" t="str">
-        <v>SPFC-C1/C2 힌지 CLOSE (SPFC-C1/C2 HINGE CLOSE)</v>
+        <v>GKFC-C1/C2 힌지 CLOSE (GKFC-C1/C2 HINGE CLOSE)</v>
       </c>
       <c r="C52" t="str">
         <v>Closed Type</v>
@@ -1911,10 +1911,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>SP-00137</v>
+        <v>GK-00137</v>
       </c>
       <c r="B53" t="str">
-        <v>SPFC-C1/C2 힌지 OPEN (SPFC-C1/C2 HINGE OPEN)</v>
+        <v>GKFC-C1/C2 힌지 OPEN (GKFC-C1/C2 HINGE OPEN)</v>
       </c>
       <c r="C53" t="str">
         <v>Opened Type</v>
@@ -1940,7 +1940,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>SP-00039</v>
+        <v>GK-00039</v>
       </c>
       <c r="B54" t="str">
         <v>라벨 스티커(제조일자 스티커)</v>
@@ -1969,10 +1969,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>SP-00138</v>
+        <v>GK-00138</v>
       </c>
       <c r="B55" t="str">
-        <v>SPFC-D1 트레이 홀더 (SPFC-D1 TRAY SUPPORTER)</v>
+        <v>GKFC-D1 트레이 홀더 (GKFC-D1 TRAY SUPPORTER)</v>
       </c>
       <c r="C55" t="str">
         <v/>
@@ -1998,7 +1998,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>SP-00139</v>
+        <v>GK-00139</v>
       </c>
       <c r="B56" t="str">
         <v>에어캡 (AIRCAP)</v>
@@ -2027,10 +2027,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>SP-00140</v>
+        <v>GK-00140</v>
       </c>
       <c r="B57" t="str">
-        <v>SPFC-C1/C2 트레이 (SPFC-C1/C2 TRAY)</v>
+        <v>GKFC-C1/C2 트레이 (GKFC-C1/C2 TRAY)</v>
       </c>
       <c r="C57" t="str">
         <v>19형 트레이</v>
@@ -2056,10 +2056,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>SP-00141</v>
+        <v>GK-00141</v>
       </c>
       <c r="B58" t="str">
-        <v>SPFC-C1/C2 트레이 커버 (SPFC-C1/C2 TRAY COVER)</v>
+        <v>GKFC-C1/C2 트레이 커버 (GKFC-C1/C2 TRAY COVER)</v>
       </c>
       <c r="C58" t="str">
         <v/>
@@ -2085,7 +2085,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>SP-00027</v>
+        <v>GK-00027</v>
       </c>
       <c r="B59" t="str">
         <v>트레이 OZ_12 SLOT_경도 90 (SPLICE HOLDER_12 SLOT_HARDNESS 90)</v>
@@ -2114,10 +2114,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>SP-00142</v>
+        <v>GK-00142</v>
       </c>
       <c r="B60" t="str">
-        <v>SPFC 인입구 마개 OD17.5 (SPFC LEADING IN ROD OD17.5 )</v>
+        <v>GKFC 인입구 마개 OD17.5 (GKFC LEADING IN ROD OD17.5 )</v>
       </c>
       <c r="C60" t="str">
         <v>17.5mm</v>
@@ -2143,10 +2143,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>SP-00143</v>
+        <v>GK-00143</v>
       </c>
       <c r="B61" t="str">
-        <v>SPFC-C1 인입구 그로멧 ID15 (SPFC-C1 CABLE GROMMET ID15)</v>
+        <v>GKFC-C1 인입구 그로멧 ID15 (GKFC-C1 CABLE GROMMET ID15)</v>
       </c>
       <c r="C61" t="str">
         <v>B-C1,C2,D1 (19,24,27) / 15mm</v>
@@ -2172,10 +2172,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>SP-00144</v>
+        <v>GK-00144</v>
       </c>
       <c r="B62" t="str">
-        <v>SPFC-D1 인입구 그로멧 ID17.5 (SPFC-D1 CABLE GROMMET ID17.5)</v>
+        <v>GKFC-D1 인입구 그로멧 ID17.5 (GKFC-D1 CABLE GROMMET ID17.5)</v>
       </c>
       <c r="C62" t="str">
         <v>B-C1,C2,D1 (19,24,27) / 17.5mm</v>
@@ -2201,10 +2201,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>SP-00145</v>
+        <v>GK-00145</v>
       </c>
       <c r="B63" t="str">
-        <v>SPFC-D1 인입구 그로멧 ID25.5 (SPFC-D1 CABLE GROMMET ID25.5)</v>
+        <v>GKFC-D1 인입구 그로멧 ID25.5 (GKFC-D1 CABLE GROMMET ID25.5)</v>
       </c>
       <c r="C63" t="str">
         <v>B-D1 (27) / 25.5mm /</v>
@@ -2230,10 +2230,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>SP-00146</v>
+        <v>GK-00146</v>
       </c>
       <c r="B64" t="str">
-        <v>PACKAGE BOX SPFC-D1 (FOR PRODUCT,NO PRINT)</v>
+        <v>PACKAGE BOX GKFC-D1 (FOR PRODUCT,NO PRINT)</v>
       </c>
       <c r="C64" t="str">
         <v>내측 : 625*315*205/NO PRINT</v>
@@ -2259,7 +2259,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>SP-00147</v>
+        <v>GK-00147</v>
       </c>
       <c r="B65" t="str">
         <v>PACKAGE BOX L-SIZE ITEM 1 (FOR SHIPPING)</v>
@@ -2288,7 +2288,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>SP-00148</v>
+        <v>GK-00148</v>
       </c>
       <c r="B66" t="str">
         <v>라벨 스티커(NBG, 상판 스티커)</v>
@@ -2317,7 +2317,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>SP-00149</v>
+        <v>GK-00149</v>
       </c>
       <c r="B67" t="str">
         <v>라벨스티커 (NBG, 상판 스티커 )</v>
@@ -2346,7 +2346,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>SP-00150</v>
+        <v>GK-00150</v>
       </c>
       <c r="B68" t="str">
         <v>실리카겔</v>
@@ -2375,7 +2375,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>SP-00151</v>
+        <v>GK-00151</v>
       </c>
       <c r="B69" t="str">
         <v>실리카겔</v>
@@ -2404,7 +2404,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>SP-00152</v>
+        <v>GK-00152</v>
       </c>
       <c r="B70" t="str">
         <v>스티로폼 120*240*5 (Styrofoam 20*240*5)</v>
@@ -2433,7 +2433,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>SP-00153</v>
+        <v>GK-00153</v>
       </c>
       <c r="B71" t="str">
         <v>스티로폼 200*240*5 (Styrofoam 200*240*5)</v>
@@ -2462,7 +2462,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>SP-00032</v>
+        <v>GK-00032</v>
       </c>
       <c r="B72" t="str">
         <v>지퍼백 W100*D150 (PLASTIC BAG W100*D150)</v>
@@ -2491,10 +2491,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>SP-00154</v>
+        <v>GK-00154</v>
       </c>
       <c r="B73" t="str">
-        <v>PACKAGE BOX SPFC-D1 (FOR PRODUCT)</v>
+        <v>PACKAGE BOX GKFC-D1 (FOR PRODUCT)</v>
       </c>
       <c r="C73" t="str">
         <v>내측 : 625*315*205/SMP</v>
@@ -2520,7 +2520,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>SP-00155</v>
+        <v>GK-00155</v>
       </c>
       <c r="B74" t="str">
         <v>PACKAGE BOX L-SIZE ITEM 1 (FOR SHIPPING, NO PRINT)</v>
@@ -2549,7 +2549,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>SP-00156</v>
+        <v>GK-00156</v>
       </c>
       <c r="B75" t="str">
         <v>PE-HOSE</v>
@@ -2578,10 +2578,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>SP-00157</v>
+        <v>GK-00157</v>
       </c>
       <c r="B76" t="str">
-        <v>SPFC-D1 MANUAL_191216</v>
+        <v>GKFC-D1 MANUAL_191216</v>
       </c>
       <c r="C76" t="str">
         <v>NBG향, 영문 매뉴얼, 210*297mm</v>
@@ -2607,7 +2607,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>SP-00005</v>
+        <v>GK-00005</v>
       </c>
       <c r="B77" t="str">
         <v>단심 열수축슬리브 L60 (SPLICE PROTECTION SLEEVE L60)</v>
@@ -2636,7 +2636,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>SP-00049</v>
+        <v>GK-00049</v>
       </c>
       <c r="B78" t="str">
         <v>T 복스 (T Handle Wrench)</v>
@@ -2665,7 +2665,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>SP-00046</v>
+        <v>GK-00046</v>
       </c>
       <c r="B79" t="str">
         <v>접지선(GROUND CABLE)</v>
@@ -2694,7 +2694,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>SP-00158</v>
+        <v>GK-00158</v>
       </c>
       <c r="B80" t="str">
         <v>보호튜브 ID8.2*OD10.2_무색_L600 (PROTECTION TUBE ID8.2*OD10.2_NC_L600)</v>
@@ -2723,7 +2723,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>SP-00159</v>
+        <v>GK-00159</v>
       </c>
       <c r="B81" t="str">
         <v>라벨 스티커(소박스 라벨)</v>
@@ -2752,7 +2752,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>SP-00160</v>
+        <v>GK-00160</v>
       </c>
       <c r="B82" t="str">
         <v>접지 러그(CABLE GROUND LUG)</v>
@@ -2781,10 +2781,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>SP-00161</v>
+        <v>GK-00161</v>
       </c>
       <c r="B83" t="str">
-        <v>SPFC-D1 인입구 그로멧 ID14-16 (SPFC-D1 CABLE GROMMET ID14-16)</v>
+        <v>GKFC-D1 인입구 그로멧 ID14-16 (GKFC-D1 CABLE GROMMET ID14-16)</v>
       </c>
       <c r="C83" t="str">
         <v>B-D1 (27) / 14-16mm</v>
@@ -2810,7 +2810,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>SP-00162</v>
+        <v>GK-00162</v>
       </c>
       <c r="B84" t="str">
         <v>보호튜브 ID4.5*OD6_무색_L850 (PROTECTION TUBE ID4.5*OD6_NC_L850)</v>
@@ -2839,7 +2839,7 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>SP-00034</v>
+        <v>GK-00034</v>
       </c>
       <c r="B85" t="str">
         <v/>
@@ -2868,7 +2868,7 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>SP-00163</v>
+        <v>GK-00163</v>
       </c>
       <c r="B86" t="str">
         <v/>

</xml_diff>